<commit_message>
update sequence dt to driver
</commit_message>
<xml_diff>
--- a/unit8_device_tree/unit8_device_tree.xlsx
+++ b/unit8_device_tree/unit8_device_tree.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Game\Linux\unit8_device_tree\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FD3B225-04AA-4450-80F1-7AC160AD8C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64EA14E1-A5F9-46A6-829C-1F3B6360FCFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{4DED5FC3-1A0F-4534-A4A0-3DE5C8B952C4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MucLuc" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,10 @@
     <sheet name="DTtoDriverMappingSequence" sheetId="7" r:id="rId5"/>
     <sheet name="deviceTree api" sheetId="8" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -7408,7 +7397,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B049B0C-149B-43FC-9295-D712528C5BE8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7419,7 +7408,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{860E8409-845C-4194-9F3A-26496BEE109C}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
@@ -7427,7 +7416,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B119285-9151-4AA2-914C-9168F431DB10}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:T178"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9864,7 +9853,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818AFC5C-713F-4650-8653-9D59B0A25DCF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M91"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10387,7 +10376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72766B5E-4D24-43F4-8273-B4BBE31EB2E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:R106"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11972,7 +11961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E393CC-C9BE-4713-8317-003849BCB02B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:BT494"/>
   <sheetFormatPr defaultColWidth="2.75" defaultRowHeight="14.25"/>
   <cols>
@@ -14352,7 +14341,7 @@
     <mergeCell ref="AA12:AD12"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B5" location="'gpio BBB'!A1" display="1.1 Device Tree Source (.dts)" xr:uid="{AF2CD107-6249-4937-9A23-4E39D12D5B20}"/>
+    <hyperlink ref="B5" location="'gpio BBB'!A1" display="1.1 Device Tree Source (.dts)" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -14360,7 +14349,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0E6175E-5182-4994-B3D9-82E30CCF48D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:BV471"/>
   <sheetFormatPr defaultColWidth="3" defaultRowHeight="14.25"/>
   <sheetData>
@@ -18151,16 +18140,16 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3:O3" location="'deviceTree api'!B31" display="1. NODE HANDLING APIs" xr:uid="{59EB1723-90C1-46F6-9E62-913F08D69B87}"/>
-    <hyperlink ref="C6:P6" location="'deviceTree api'!B70" display="2. PROPERTY READING APIs" xr:uid="{46F04302-E2AD-447F-9A4B-9104C3010990}"/>
-    <hyperlink ref="C10:S10" location="'deviceTree api'!B124" display="3. RESOURCE MANAGEMENT APIs" xr:uid="{CF7F4E4D-6892-4854-9BC9-1EC6FF33BE57}"/>
-    <hyperlink ref="C13:R13" location="'deviceTree api'!B168" display="4. CLOCK MANAGEMENT APIs" xr:uid="{40108E0E-C728-4F81-B8C5-8CB025210C96}"/>
-    <hyperlink ref="C15:I15" location="'deviceTree api'!B216" display="5. GPIO APIs" xr:uid="{CDC30919-12D8-4ED5-9147-2B10397B8894}"/>
-    <hyperlink ref="C17:M17" location="'deviceTree api'!B262" display="6. PINCONTROL APIs" xr:uid="{AB0C68E2-7242-46B3-96A8-C160040BB60B}"/>
-    <hyperlink ref="C21:P21" location="'deviceTree api'!B350" display="8. DEVICE MATCHING APIs" xr:uid="{90EEC3EC-6F2F-4608-AD75-0EFE69EDFC79}"/>
-    <hyperlink ref="C23:Q23" location="'deviceTree api'!B379" display="9. CHILD NODE ITERATION" xr:uid="{739DD18D-4D7C-4BAF-AC78-AF5707B69BAC}"/>
-    <hyperlink ref="C19:R19" location="'deviceTree api'!B329" display="7. PHANDLE &amp; REFERENCE APIs" xr:uid="{D1A5727A-8D0E-4670-85EA-0B18F5991A9B}"/>
-    <hyperlink ref="C25:Y25" location="'deviceTree api'!B423" display="10. BEST PRACTICES &amp; COMMON PATTERNS" xr:uid="{F5140593-C2E7-4198-B58A-A4DB0CBCAFA8}"/>
+    <hyperlink ref="C3:O3" location="'deviceTree api'!B31" display="1. NODE HANDLING APIs" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="C6:P6" location="'deviceTree api'!B70" display="2. PROPERTY READING APIs" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
+    <hyperlink ref="C10:S10" location="'deviceTree api'!B124" display="3. RESOURCE MANAGEMENT APIs" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="C13:R13" location="'deviceTree api'!B168" display="4. CLOCK MANAGEMENT APIs" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
+    <hyperlink ref="C15:I15" location="'deviceTree api'!B216" display="5. GPIO APIs" xr:uid="{00000000-0004-0000-0500-000004000000}"/>
+    <hyperlink ref="C17:M17" location="'deviceTree api'!B262" display="6. PINCONTROL APIs" xr:uid="{00000000-0004-0000-0500-000005000000}"/>
+    <hyperlink ref="C21:P21" location="'deviceTree api'!B350" display="8. DEVICE MATCHING APIs" xr:uid="{00000000-0004-0000-0500-000006000000}"/>
+    <hyperlink ref="C23:Q23" location="'deviceTree api'!B379" display="9. CHILD NODE ITERATION" xr:uid="{00000000-0004-0000-0500-000007000000}"/>
+    <hyperlink ref="C19:R19" location="'deviceTree api'!B329" display="7. PHANDLE &amp; REFERENCE APIs" xr:uid="{00000000-0004-0000-0500-000008000000}"/>
+    <hyperlink ref="C25:Y25" location="'deviceTree api'!B423" display="10. BEST PRACTICES &amp; COMMON PATTERNS" xr:uid="{00000000-0004-0000-0500-000009000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>